<commit_message>
Remove the last integration gaps: admin role from profiles, one-step add part and pull-to-refresh on the phone
The website reads profiles.role at login (email list only as a fallback). The
mobile app adds parts through the add_booking_part database function, the same
as the website, and the bookings list and booking page reload when pulled down.
Documents, tracker, forms, SRS v3.0 and evidence updated to match.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pyu1PuNoiQSXEChGBbiq3J
</commit_message>
<xml_diff>
--- a/project-docs/phase-3/tracker/Group Y - ITC327W Phase 3 Project Progress Tracker (updated 30 Oct).xlsx
+++ b/project-docs/phase-3/tracker/Group Y - ITC327W Phase 3 Project Progress Tracker (updated 30 Oct).xlsx
@@ -716,7 +716,7 @@
       </x:c>
       <x:c r="E5" s="46" t="n">
         <x:f>COUNTIF('Development Progress'!G4:G33,"Completed")</x:f>
-        <x:v>11</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -729,7 +729,7 @@
       </x:c>
       <x:c r="E6" s="46" t="n">
         <x:f>COUNTIF('Development Progress'!G4:G33,"In Progress")</x:f>
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -759,7 +759,7 @@
       </x:c>
       <x:c r="E8" s="47" t="n">
         <x:f>IFERROR(AVERAGE('Development Progress'!H4:H33),0)</x:f>
-        <x:v>0.79</x:v>
+        <x:v>0.878</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1012,18 +1012,20 @@
       <x:c r="E7" s="34" t="str">
         <x:v>2026-10-25</x:v>
       </x:c>
-      <x:c r="F7" s="34"/>
+      <x:c r="F7" s="34" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
       <x:c r="G7" s="34" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="H7" s="54" t="n">
-        <x:v>0.9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I7" s="34" t="str">
         <x:v>mobile/lib/features/*/data</x:v>
       </x:c>
       <x:c r="J7" s="34" t="str">
-        <x:v>All main functions read/write Supabase and ran against the live project 30 Oct. Done: Send on WhatsApp, kIsWeb guard, missing logo asset added, dead home_screen.dart removed. Still open: pull-to-refresh on staff lists (P3-25) and add part through add_booking_part (limitation L6).</x:v>
+        <x:v>All main functions read/write Supabase and ran against the live project 30 Oct. Done: Send on WhatsApp, kIsWeb guard, missing logo asset, pull-to-refresh on the bookings list and booking page, add part through the add_booking_part database function (tested: part saved, stock 3 to 2, one stock movement).</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1074,18 +1076,20 @@
       <x:c r="E9" s="34" t="str">
         <x:v>2026-10-25</x:v>
       </x:c>
-      <x:c r="F9" s="34"/>
+      <x:c r="F9" s="34" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
       <x:c r="G9" s="34" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="H9" s="54" t="n">
-        <x:v>0.95</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I9" s="34" t="str">
         <x:v>web/Pages, web/Services</x:v>
       </x:c>
       <x:c r="J9" s="34" t="str">
-        <x:v>All main functions use Supabase and were run live 30 Oct (16 screenshots). 30 Oct: labour now read and written from booking_labor, the same table as the phone. Open: admin role still read from an email list instead of profiles (P3-20).</x:v>
+        <x:v>All main functions use Supabase and were run live 30 Oct (16 screenshots). Labour read and written from booking_labor; admin role read from profiles.role at login (checked with the email list emptied: admin still sees Finalize, mechanic does not).</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1168,18 +1172,20 @@
       <x:c r="E12" s="34" t="str">
         <x:v>2026-10-25</x:v>
       </x:c>
-      <x:c r="F12" s="34"/>
+      <x:c r="F12" s="34" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
       <x:c r="G12" s="34" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="H12" s="54" t="n">
-        <x:v>0.95</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I12" s="34" t="str">
         <x:v>project-docs/phase-3/unit-4-readiness.md section 4</x:v>
       </x:c>
       <x:c r="J12" s="34" t="str">
-        <x:v>Status, phase, reference code and invoice number match in both apps. Labour decided 30 Oct: one ledger, booking_labor (PR #21), tested R350 + R150 = R500 on page and invoice. Open: admin role read from two places.</x:v>
+        <x:v>Status, phase, reference code, invoice number, labour and the admin role now come from the same data in both apps. Tested 30 Oct.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1508,16 +1514,18 @@
       <x:c r="E23" s="34" t="str">
         <x:v>2026-10-25</x:v>
       </x:c>
-      <x:c r="F23" s="34"/>
+      <x:c r="F23" s="34" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
       <x:c r="G23" s="34" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="H23" s="54" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I23" s="34"/>
       <x:c r="J23" s="34" t="str">
-        <x:v>Still open: web reads the admin role from an email list (AdminEmails), the phone from profiles.role.</x:v>
+        <x:v>Done 30 Oct: the website reads profiles.role at login (falls back to the email list only if the profile cannot be read).</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1660,18 +1668,20 @@
       <x:c r="E28" s="34" t="str">
         <x:v>2026-10-24</x:v>
       </x:c>
-      <x:c r="F28" s="34"/>
+      <x:c r="F28" s="34" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
       <x:c r="G28" s="34" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="H28" s="54" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I28" s="34" t="str">
         <x:v>project-docs/phase-3/code-guide.md Part 2 Step 3</x:v>
       </x:c>
       <x:c r="J28" s="34" t="str">
-        <x:v>Still missing in Gary's app on 30 Oct (checked): a web change shows after reload only. Needed to see web changes live on the phone.</x:v>
+        <x:v>Done 30 Oct: RefreshIndicator on the bookings list and the booking page; tested (a phase changed in the database showed after pulling down, m27).</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2306,21 +2316,35 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="34" t="str"/>
-      <x:c r="B18" s="34" t="str"/>
-      <x:c r="C18" s="34" t="str"/>
-      <x:c r="D18" s="34" t="str"/>
-      <x:c r="E18" s="34" t="str"/>
-      <x:c r="F18" s="34" t="str"/>
+      <x:c r="A18" s="34" t="str">
+        <x:v>Wisani Nkuna</x:v>
+      </x:c>
+      <x:c r="B18" s="34" t="str">
+        <x:v>222010787</x:v>
+      </x:c>
+      <x:c r="C18" s="34" t="str">
+        <x:v>Integration</x:v>
+      </x:c>
+      <x:c r="D18" s="34" t="str">
+        <x:v>Remove the last integration gaps</x:v>
+      </x:c>
+      <x:c r="E18" s="34" t="str">
+        <x:v>Website admin role from profiles.role; phone add part through add_booking_part; pull-to-refresh on the phone lists and booking page; tested live</x:v>
+      </x:c>
+      <x:c r="F18" s="34" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
       <x:c r="G18" s="34" t="str"/>
-      <x:c r="H18" s="34" t="str"/>
+      <x:c r="H18" s="34" t="str">
+        <x:v>web/Auth/AdminAccess.cs; mobile/lib/features/bookings</x:v>
+      </x:c>
       <x:c r="I18" s="34" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="J18" s="34" t="str"/>
       <x:c r="K18" s="34" t="str"/>
       <x:c r="L18" s="34" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -3060,7 +3084,7 @@
         <x:v>project-docs/phase-3/evidence (m09-m16, w04, m24); recording pending (Kea)</x:v>
       </x:c>
       <x:c r="I4" s="34" t="str">
-        <x:v>Shown working both directions 30 Oct. Web add part uses add_booking_part; mobile still makes three calls. Flutter needs a reload to show web changes.</x:v>
+        <x:v>Shown working both directions 30 Oct. Both apps add a part through add_booking_part. Pull down on the phone to see web changes (m27).</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -3116,7 +3140,7 @@
       </x:c>
       <x:c r="H6" s="34" t="str"/>
       <x:c r="I6" s="34" t="str">
-        <x:v>Phone and web show the same stock (m23, w06; 3 to 2 when the part was added, back to 3 after the test booking was deleted). Mobile add part is still three calls.</x:v>
+        <x:v>Phone and web show the same stock (m23, w06; 3 to 2 when the part was added, back to 3 after the test booking was deleted). Both apps add parts through add_booking_part.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4083,10 +4107,14 @@
         <x:v>2026-10-25</x:v>
       </x:c>
       <x:c r="G7" s="34" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="H7" s="34" t="str"/>
-      <x:c r="I7" s="34" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="H7" s="34" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="I7" s="34" t="str">
+        <x:v>Done 30 Oct: the website reads profiles.role at login.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="34" t="str">
@@ -4137,10 +4165,14 @@
         <x:v>2026-10-25</x:v>
       </x:c>
       <x:c r="G9" s="34" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="H9" s="34" t="str"/>
-      <x:c r="I9" s="34" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="H9" s="34" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="I9" s="34" t="str">
+        <x:v>Done 30 Oct: the phone now calls add_booking_part; tested.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="34" t="str">
@@ -4224,7 +4256,7 @@
         <x:v>2026-10-18</x:v>
       </x:c>
       <x:c r="I12" s="34" t="str">
-        <x:v>Known limitation; the web dashboard does live-reload.</x:v>
+        <x:v>Known limitation; the web dashboard live-reloads and the phone reloads when pulled down (m27).</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4359,11 +4391,13 @@
         <x:v>2026-10-24</x:v>
       </x:c>
       <x:c r="G17" s="34" t="str">
-        <x:v>Not Started</x:v>
-      </x:c>
-      <x:c r="H17" s="34" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="H17" s="34" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
       <x:c r="I17" s="34" t="str">
-        <x:v>Still open 30 Oct: no pull-to-refresh in Gary's app; reload to see web changes.</x:v>
+        <x:v>Done 30 Oct: pull-to-refresh on the bookings list and booking page (m27).</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -4522,7 +4556,7 @@
         <x:v>Someone could be admin in one app only</x:v>
       </x:c>
       <x:c r="D23" s="34" t="str">
-        <x:v>Web to read profiles.role (P3-20)</x:v>
+        <x:v>The website reads profiles.role at login (done 30 Oct)</x:v>
       </x:c>
       <x:c r="E23" s="34" t="str">
         <x:v>Wisani Nkuna</x:v>
@@ -4531,11 +4565,13 @@
         <x:v>2026-11-02</x:v>
       </x:c>
       <x:c r="G23" s="34" t="str">
-        <x:v>In Progress</x:v>
-      </x:c>
-      <x:c r="H23" s="34" t="str"/>
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="H23" s="34" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
       <x:c r="I23" s="34" t="str">
-        <x:v>Open known limitation.</x:v>
+        <x:v>Fixed 30 Oct, tested with the email list emptied.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -4746,7 +4782,7 @@
         <x:v>What was completed during Phase 3?</x:v>
       </x:c>
       <x:c r="B5" s="34" t="str">
-        <x:v>Both apps run on one shared Supabase project and were run live on 30 Oct. Since 20 Oct: web restyled to match the mobile app and redeployed from main; Gary's WhatsApp sheet and fingerprint login merged; migrations 0009-0011 run; one labour ledger; 26 mobile and 16 web screenshots; SRS v3.0; submission ZIP.</x:v>
+        <x:v>Both apps run on one shared Supabase project and were run live on 30 Oct. Since 20 Oct: web restyled to match the mobile app and redeployed from main; Gary's WhatsApp sheet and fingerprint login merged; migrations 0009-0011 run; one labour ledger; 26 mobile and 16 web screenshots; SRS v3.0; submission ZIP. Also 30 Oct: pull-to-refresh and one-step add part on the phone, admin role from profiles on the website.</x:v>
       </x:c>
       <x:c r="C5" s="34"/>
       <x:c r="E5" t="str">
@@ -4761,7 +4797,7 @@
         <x:v>Which functions or processes remain incomplete?</x:v>
       </x:c>
       <x:c r="B6" s="34" t="str">
-        <x:v>Pull-to-refresh and add part through the database function in the mobile app; web admin role from profiles; recording of P1 and P2; retaking three screenshots after the labour change; push notifications and fingerprint login on a real phone.</x:v>
+        <x:v>Recording of P1 and P2; push notifications and fingerprint login on a real phone; the Firebase key must still be revoked.</x:v>
       </x:c>
       <x:c r="C6" s="34"/>
       <x:c r="E6" t="str">
@@ -4776,7 +4812,7 @@
         <x:v>What known limitations remain?</x:v>
       </x:c>
       <x:c r="B7" s="34" t="str">
-        <x:v>Phone does not update live (reload needed); push Android only; Vercel container sleeps when idle; mobile add part is three calls; admin role in two places; Firebase key still to be revoked.</x:v>
+        <x:v>Phone does not update live (pull down to reload); push Android only; Vercel container sleeps when idle; the Firebase key is still valid until revoked.</x:v>
       </x:c>
       <x:c r="C7" s="34"/>
       <x:c r="E7" t="str">

</xml_diff>